<commit_message>
feat: I6 통계 대시보드·S5 내 통계 (Chart.js, group by 집계)
</commit_message>
<xml_diff>
--- a/docs/AssignHub_요구사항정의서_ERD.xlsx
+++ b/docs/AssignHub_요구사항정의서_ERD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\assignhub\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AD6D298-53C4-49D1-A545-C1BDC09816A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915662C1-C5FB-458D-9312-CAED39DC31A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C867C853-1BD9-4C61-8B6E-EBEFC9874430}"/>
+    <workbookView xWindow="3465" yWindow="2250" windowWidth="21600" windowHeight="11295" xr2:uid="{C867C853-1BD9-4C61-8B6E-EBEFC9874430}"/>
   </bookViews>
   <sheets>
     <sheet name="개요" sheetId="1" r:id="rId1"/>
@@ -155,9 +155,6 @@
     <t>W2</t>
   </si>
   <si>
-    <t>예정</t>
-  </si>
-  <si>
     <t>I2</t>
   </si>
   <si>
@@ -1050,6 +1047,10 @@
   </si>
   <si>
     <t>• 테이블 관계와 필수 컬럼은 수업 제공 ERD를 따르며, 컬럼을 추가하면 README에 이유를 기록합니다.</t>
+  </si>
+  <si>
+    <t>완료</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>완료</t>
@@ -1504,14 +1505,14 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5668,139 +5669,139 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="50" t="s">
-        <v>312</v>
-      </c>
-      <c r="B4" s="62" t="s">
-        <v>243</v>
-      </c>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
+        <v>311</v>
+      </c>
+      <c r="B4" s="61" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
     </row>
     <row r="5" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" s="60" t="s">
         <v>313</v>
       </c>
-      <c r="B5" s="61" t="s">
-        <v>314</v>
-      </c>
-      <c r="C5" s="61"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
     </row>
     <row r="6" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52" t="s">
+        <v>314</v>
+      </c>
+      <c r="B6" s="62" t="s">
         <v>315</v>
       </c>
-      <c r="B6" s="60" t="s">
-        <v>316</v>
-      </c>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
     </row>
     <row r="7" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="51" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="61" t="s">
-        <v>317</v>
-      </c>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
+        <v>143</v>
+      </c>
+      <c r="B7" s="60" t="s">
+        <v>316</v>
+      </c>
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
     </row>
     <row r="8" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="52" t="s">
+        <v>317</v>
+      </c>
+      <c r="B8" s="62" t="s">
         <v>318</v>
       </c>
-      <c r="B8" s="60" t="s">
-        <v>319</v>
-      </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
     </row>
     <row r="9" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="51" t="s">
+        <v>319</v>
+      </c>
+      <c r="B9" s="60" t="s">
         <v>320</v>
       </c>
-      <c r="B9" s="61" t="s">
-        <v>321</v>
-      </c>
-      <c r="C9" s="61"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="61"/>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
     </row>
     <row r="10" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="52" t="s">
+        <v>321</v>
+      </c>
+      <c r="B10" s="62" t="s">
         <v>322</v>
       </c>
-      <c r="B10" s="60" t="s">
-        <v>323</v>
-      </c>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
     </row>
     <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="51" t="s">
-        <v>146</v>
-      </c>
-      <c r="B11" s="61" t="s">
-        <v>324</v>
-      </c>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
+        <v>145</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>323</v>
+      </c>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
     </row>
     <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="52" t="s">
+        <v>324</v>
+      </c>
+      <c r="B12" s="62" t="s">
         <v>325</v>
       </c>
-      <c r="B12" s="60" t="s">
-        <v>326</v>
-      </c>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
     </row>
     <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="51" t="s">
+        <v>326</v>
+      </c>
+      <c r="B13" s="60" t="s">
         <v>327</v>
       </c>
-      <c r="B13" s="61" t="s">
-        <v>328</v>
-      </c>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="61"/>
+      <c r="C13" s="60"/>
+      <c r="D13" s="60"/>
+      <c r="E13" s="60"/>
     </row>
     <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="52" t="s">
+        <v>328</v>
+      </c>
+      <c r="B14" s="62" t="s">
         <v>329</v>
       </c>
-      <c r="B14" s="60" t="s">
-        <v>330</v>
-      </c>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
     </row>
     <row r="16" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A16" s="49" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5808,13 +5809,13 @@
         <v>3</v>
       </c>
       <c r="B17" s="50" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C17" s="50" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="50" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -5844,16 +5845,16 @@
       </c>
       <c r="C19" s="54">
         <f>COUNTIFS(요구사항정의서!$B$5:$B$100,A19,요구사항정의서!$I$5:$I$100,"완료")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D19" s="57">
         <f>IF(B19=0,0,C19/B19)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="53">
         <f>COUNTIF(요구사항정의서!$B$5:$B$100,A20)</f>
@@ -5861,16 +5862,16 @@
       </c>
       <c r="C20" s="53">
         <f>COUNTIFS(요구사항정의서!$B$5:$B$100,A20,요구사항정의서!$I$5:$I$100,"완료")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" s="56">
         <f>IF(B20=0,0,C20/B20)</f>
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="55" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B21" s="55">
         <f>SUM(B18:B20)</f>
@@ -5878,46 +5879,46 @@
       </c>
       <c r="C21" s="55">
         <f>SUM(C18:C20)</f>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D21" s="58">
         <f>IF(B21=0,0,C21/B21)</f>
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A23" s="49" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="59" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="59" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="59" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="D18:D21">
@@ -6160,297 +6161,297 @@
         <v>39</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="F10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>39</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>39</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="H12" s="9" t="s">
-        <v>58</v>
-      </c>
       <c r="I12" s="9" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="16" t="s">
         <v>34</v>
       </c>
       <c r="C13" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>64</v>
-      </c>
       <c r="H13" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="E14" s="9" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="H14" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="H14" s="9" t="s">
-        <v>70</v>
-      </c>
       <c r="I14" s="9" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="D15" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>74</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>76</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>39</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C16" s="13" t="s">
+      <c r="D16" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="F16" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>39</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="27" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="F17" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>87</v>
-      </c>
       <c r="G17" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="13" t="s">
+      <c r="D18" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>15</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="12" t="s">
+      <c r="D19" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>15</v>
       </c>
       <c r="F19" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>96</v>
-      </c>
       <c r="H19" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>40</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -6493,193 +6494,193 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="8.1" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>122</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="F10" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="C12" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>140</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -6707,30 +6708,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6738,16 +6739,16 @@
         <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="8" t="s">
         <v>150</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6755,16 +6756,16 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6772,16 +6773,16 @@
         <v>34</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>155</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>156</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6789,16 +6790,16 @@
         <v>34</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>52</v>
-      </c>
       <c r="E8" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6806,16 +6807,16 @@
         <v>34</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6823,16 +6824,16 @@
         <v>34</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>64</v>
-      </c>
       <c r="E10" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6840,67 +6841,67 @@
         <v>34</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>69</v>
-      </c>
       <c r="E11" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>76</v>
-      </c>
       <c r="E12" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -6908,13 +6909,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>25</v>
@@ -6945,138 +6946,138 @@
   <sheetData>
     <row r="1" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="8.1" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="37" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A37" s="49" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="C38" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="D38" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="E38" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="E38" s="6" t="s">
-        <v>289</v>
-      </c>
       <c r="F38" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>291</v>
       </c>
-      <c r="C39" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="D39" s="8" t="s">
+      <c r="E39" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="F39" s="5" t="s">
         <v>293</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="E40" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="E40" s="7" t="s">
+      <c r="F40" s="7" t="s">
         <v>296</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="B41" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>299</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="D41" s="8" t="s">
+      <c r="E41" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="F41" s="5" t="s">
         <v>301</v>
-      </c>
-      <c r="F41" s="5" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="E42" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="E42" s="7" t="s">
+      <c r="F42" s="7" t="s">
         <v>304</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="B43" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="C43" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="C43" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="E43" s="5" t="s">
+      <c r="F43" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -7108,1075 +7109,1075 @@
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="8.1" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="C4" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="D4" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="E4" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="F4" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="G4" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="H4" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="I4" s="24" t="s">
         <v>177</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="J4" s="24" t="s">
         <v>178</v>
-      </c>
-      <c r="J4" s="24" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="F5" s="20" t="s">
-        <v>185</v>
-      </c>
       <c r="G5" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="64"/>
       <c r="B6" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>192</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="64"/>
       <c r="B7" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="D7" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="64"/>
       <c r="B8" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="D8" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>202</v>
-      </c>
       <c r="F8" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G8" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>187</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="64"/>
       <c r="B9" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="D9" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="F9" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J9" s="5" t="s">
         <v>207</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="64"/>
       <c r="B10" s="35" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="36" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="D10" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="G10" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="H10" s="35" t="s">
+        <v>186</v>
+      </c>
+      <c r="I10" s="35" t="s">
+        <v>185</v>
+      </c>
+      <c r="J10" s="37" t="s">
         <v>210</v>
-      </c>
-      <c r="D10" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>206</v>
-      </c>
-      <c r="F10" s="38" t="s">
-        <v>186</v>
-      </c>
-      <c r="G10" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="H10" s="35" t="s">
-        <v>187</v>
-      </c>
-      <c r="I10" s="35" t="s">
-        <v>186</v>
-      </c>
-      <c r="J10" s="37" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="65" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>181</v>
+      </c>
+      <c r="D11" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="B11" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>182</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>213</v>
-      </c>
       <c r="E11" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="F11" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="F11" s="33" t="s">
-        <v>185</v>
-      </c>
       <c r="G11" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="H11" s="30" t="s">
         <v>186</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="I11" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="J11" s="32" t="s">
         <v>187</v>
-      </c>
-      <c r="I11" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="J11" s="32" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="64"/>
       <c r="B12" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G12" s="23" t="s">
         <v>215</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="F12" s="21" t="s">
+      <c r="H12" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="I12" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="J12" s="7" t="s">
         <v>216</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="64"/>
       <c r="B13" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F13" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G13" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>187</v>
-      </c>
       <c r="I13" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="64"/>
       <c r="B14" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C14" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="J14" s="7" t="s">
         <v>220</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="64"/>
       <c r="B15" s="45" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C15" s="46" t="s">
+        <v>221</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>224</v>
-      </c>
       <c r="F15" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="G15" s="48" t="s">
+        <v>185</v>
+      </c>
+      <c r="H15" s="45" t="s">
         <v>186</v>
       </c>
-      <c r="G15" s="48" t="s">
-        <v>186</v>
-      </c>
-      <c r="H15" s="45" t="s">
-        <v>187</v>
-      </c>
       <c r="I15" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="65" t="s">
+        <v>224</v>
+      </c>
+      <c r="B16" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" s="42" t="s">
         <v>225</v>
       </c>
-      <c r="B16" s="40" t="s">
-        <v>181</v>
-      </c>
-      <c r="C16" s="41" t="s">
-        <v>182</v>
-      </c>
-      <c r="D16" s="42" t="s">
-        <v>226</v>
-      </c>
       <c r="E16" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="F16" s="43" t="s">
         <v>184</v>
       </c>
-      <c r="F16" s="43" t="s">
-        <v>185</v>
-      </c>
       <c r="G16" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="H16" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="H16" s="40" t="s">
+      <c r="I16" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="J16" s="42" t="s">
         <v>187</v>
-      </c>
-      <c r="I16" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="J16" s="42" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="64"/>
       <c r="B17" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C17" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G17" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="F17" s="20" t="s">
+      <c r="H17" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="I17" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="I17" s="8" t="s">
+      <c r="J17" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="64"/>
       <c r="B18" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C18" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="J18" s="7" t="s">
         <v>232</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>216</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="64"/>
       <c r="B19" s="45" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C19" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>235</v>
-      </c>
       <c r="E19" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F19" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="G19" s="48" t="s">
+        <v>185</v>
+      </c>
+      <c r="H19" s="45" t="s">
         <v>186</v>
       </c>
-      <c r="G19" s="48" t="s">
-        <v>186</v>
-      </c>
-      <c r="H19" s="45" t="s">
-        <v>187</v>
-      </c>
       <c r="I19" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="65" t="s">
+        <v>235</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>181</v>
+      </c>
+      <c r="D20" s="42" t="s">
         <v>236</v>
       </c>
-      <c r="B20" s="40" t="s">
-        <v>181</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>182</v>
-      </c>
-      <c r="D20" s="42" t="s">
-        <v>237</v>
-      </c>
       <c r="E20" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="F20" s="43" t="s">
         <v>184</v>
       </c>
-      <c r="F20" s="43" t="s">
-        <v>185</v>
-      </c>
       <c r="G20" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="H20" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="H20" s="40" t="s">
+      <c r="I20" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="J20" s="42" t="s">
         <v>187</v>
-      </c>
-      <c r="I20" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="J20" s="42" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="64"/>
       <c r="B21" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C21" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G21" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="F21" s="20" t="s">
+      <c r="H21" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G21" s="22" t="s">
-        <v>229</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>187</v>
-      </c>
       <c r="I21" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="64"/>
       <c r="B22" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C22" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="E22" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>241</v>
-      </c>
       <c r="F22" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G22" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H22" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G22" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>187</v>
-      </c>
       <c r="I22" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="64"/>
       <c r="B23" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C23" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="E23" s="5" t="s">
-        <v>244</v>
-      </c>
       <c r="F23" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H23" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G23" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>187</v>
-      </c>
       <c r="I23" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="64"/>
       <c r="B24" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C24" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="E24" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F24" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="J24" s="7" t="s">
         <v>246</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="F24" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I24" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="64"/>
       <c r="B25" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C25" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="J25" s="5" t="s">
         <v>249</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="F25" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="G25" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="64"/>
       <c r="B26" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="D26" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="E26" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="J26" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="F26" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I26" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="64"/>
       <c r="B27" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>256</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="D27" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>259</v>
-      </c>
       <c r="F27" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="64"/>
       <c r="B28" s="35" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F28" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="H28" s="35" t="s">
         <v>186</v>
       </c>
-      <c r="G28" s="39" t="s">
-        <v>186</v>
-      </c>
-      <c r="H28" s="35" t="s">
-        <v>187</v>
-      </c>
       <c r="I28" s="35" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="65" t="s">
+        <v>260</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>180</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>181</v>
+      </c>
+      <c r="D29" s="32" t="s">
         <v>261</v>
       </c>
-      <c r="B29" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>182</v>
-      </c>
-      <c r="D29" s="32" t="s">
-        <v>262</v>
-      </c>
       <c r="E29" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="F29" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="F29" s="33" t="s">
-        <v>185</v>
-      </c>
       <c r="G29" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="H29" s="30" t="s">
         <v>186</v>
       </c>
-      <c r="H29" s="30" t="s">
+      <c r="I29" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="J29" s="32" t="s">
         <v>187</v>
-      </c>
-      <c r="I29" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="J29" s="32" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="64"/>
       <c r="B30" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C30" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="E30" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G30" s="23" t="s">
         <v>264</v>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="F30" s="21" t="s">
+      <c r="H30" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="I30" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="J30" s="7" t="s">
         <v>265</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I30" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="64"/>
       <c r="B31" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F31" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="H31" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G31" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>187</v>
-      </c>
       <c r="I31" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="64"/>
       <c r="B32" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F32" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G32" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G32" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>187</v>
-      </c>
       <c r="I32" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="64"/>
       <c r="B33" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C33" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="E33" s="5" t="s">
-        <v>259</v>
-      </c>
       <c r="F33" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="64"/>
       <c r="B34" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C34" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="E34" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F34" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G34" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="I34" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="J34" s="7" t="s">
         <v>270</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="F34" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G34" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="J34" s="7" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="64"/>
       <c r="B35" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F35" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="H35" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="G35" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H35" s="8" t="s">
-        <v>187</v>
-      </c>
       <c r="I35" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="64"/>
       <c r="B36" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C36" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="E36" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="F36" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="I36" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="J36" s="7" t="s">
         <v>275</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="I36" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="J36" s="7" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="64"/>
       <c r="B37" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C37" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>278</v>
-      </c>
       <c r="E37" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="66"/>
       <c r="B38" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="C38" s="26" t="s">
         <v>279</v>
       </c>
-      <c r="C38" s="26" t="s">
+      <c r="D38" s="27" t="s">
         <v>280</v>
       </c>
-      <c r="D38" s="27" t="s">
-        <v>281</v>
-      </c>
       <c r="E38" s="27" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F38" s="28" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G38" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H38" s="25" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I38" s="25" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J38" s="27" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>